<commit_message>
implementacion exportacion a jira csv
</commit_message>
<xml_diff>
--- a/input/HU-123 - Matriz de Casos.xlsx
+++ b/input/HU-123 - Matriz de Casos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willi\Personal\Proyects\Python\aut-excel-to-word\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{524AD665-7341-4709-B35A-74CFC4365E69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC0108C9-F285-4BB2-9ADA-F48E3BFD4379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,13 +57,6 @@
     <t>Pasos</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Navegue hasta la URL de la aplicación
-2) Navegue hasta la URL de la aplicación.
-3) Introduzca el nombre de usuario.
-4) Introduzca la contraseña
-5) Haga clic en el botón de inicio de sesión </t>
-  </si>
-  <si>
     <t>Usuario: abc@mail.com 
 Contraseña: Pass1</t>
   </si>
@@ -79,6 +72,13 @@
   </si>
   <si>
     <t>TC_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Navegue hasta la URL de la aplicación
+2) Navegue hasta la URL de la aplicación
+3) Introduzca el nombre de usuario
+4) Introduzca la contraseña
+5) Haga clic en el botón de inicio de sesión </t>
   </si>
 </sst>
 </file>
@@ -469,10 +469,10 @@
         <v>4</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>5</v>
@@ -480,16 +480,16 @@
     </row>
     <row r="4" spans="2:6" ht="57" x14ac:dyDescent="0.45">
       <c r="B4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>13</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
Sanitizar texto para word
</commit_message>
<xml_diff>
--- a/input/HU-123 - Matriz de Casos.xlsx
+++ b/input/HU-123 - Matriz de Casos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willi\Personal\Proyects\Python\aut-excel-to-word\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC0108C9-F285-4BB2-9ADA-F48E3BFD4379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97B90978-096D-4BAC-8E2D-90FD046E708C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,10 +57,6 @@
     <t>Pasos</t>
   </si>
   <si>
-    <t>Usuario: abc@mail.com 
-Contraseña: Pass1</t>
-  </si>
-  <si>
     <t>Usuario: xyz@mail.com 
 Contraseña: Pass1</t>
   </si>
@@ -74,11 +70,14 @@
     <t>TC_002</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Navegue hasta la URL de la aplicación
-2) Navegue hasta la URL de la aplicación
-3) Introduzca el nombre de usuario
-4) Introduzca la contraseña
-5) Haga clic en el botón de inicio de sesión </t>
+    <t xml:space="preserve">1) Navegue hasta la URL de la aplicación 
+2) Introduzca el nombre de usuario
+3) Introduzca la contraseña
+4) Haga clic en el botón de inicio de sesión </t>
+  </si>
+  <si>
+    <t>Usuario: abc@mail.com 
+Contraseña: &lt;pass&gt;</t>
   </si>
 </sst>
 </file>
@@ -461,7 +460,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="2:6" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:6" ht="57" x14ac:dyDescent="0.45">
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
@@ -469,10 +468,10 @@
         <v>4</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>5</v>
@@ -480,16 +479,16 @@
     </row>
     <row r="4" spans="2:6" ht="57" x14ac:dyDescent="0.45">
       <c r="B4" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
Metodos mejorados y abstraidos
</commit_message>
<xml_diff>
--- a/input/HU-123 - Matriz de Casos.xlsx
+++ b/input/HU-123 - Matriz de Casos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willi\Personal\Proyects\Python\aut-excel-to-word\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97B90978-096D-4BAC-8E2D-90FD046E708C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36143ECC-C9EB-425D-A5EA-906907B89373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,9 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
-    <t>ID de caso de prueba</t>
-  </si>
-  <si>
     <t>Descripción de la prueba</t>
   </si>
   <si>
@@ -78,6 +75,9 @@
   <si>
     <t>Usuario: abc@mail.com 
 Contraseña: &lt;pass&gt;</t>
+  </si>
+  <si>
+    <t>ID del caso</t>
   </si>
 </sst>
 </file>
@@ -445,53 +445,53 @@
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>2</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="57" x14ac:dyDescent="0.45">
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>4</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" spans="2:6" ht="57" x14ac:dyDescent="0.45">
       <c r="B4" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="F4" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
resultados esperado por cada paso
</commit_message>
<xml_diff>
--- a/input/HU-123 - Matriz de Casos.xlsx
+++ b/input/HU-123 - Matriz de Casos.xlsx
@@ -1,24 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29512"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willi\Personal\Proyects\Python\aut-excel-to-word\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7939ACF2-AA5F-45BF-9923-92A071F8F00E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{7939ACF2-AA5F-45BF-9923-92A071F8F00E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ADFE17CC-4964-4AE7-A62C-B9BAE8A1AAC3}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -27,28 +38,47 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
+    <t>ID del caso</t>
+  </si>
+  <si>
     <t>Descripción de la prueba</t>
   </si>
   <si>
     <t>Prerrequisitos</t>
   </si>
   <si>
+    <t>Pasos</t>
+  </si>
+  <si>
     <t>Resultado esperado</t>
   </si>
   <si>
+    <t>TC_001</t>
+  </si>
+  <si>
     <t>Verificar que los usuarios puedan iniciar sesión correctamente usando un correo electrónico y una contraseña válidos</t>
   </si>
   <si>
-    <t>Se debe mostrar el panel de control de la cuenta de usuario.</t>
+    <t>Usuario: abc@mail.com 
+Contraseña: &lt;pass&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Navegue hasta la URL de la aplicación 
+2) Introduzca el nombre de usuario
+3) Introduzca la contraseña
+4) Haga clic en el botón de inicio de sesión </t>
+  </si>
+  <si>
+    <t>1) Se visualiza la pantalla de Login
+2) Se visualiza el nombre de usuario
+3) Se visualiza la contraseña enmascarada
+4) Se debe mostrar el panel de control de la cuenta de usuario.</t>
+  </si>
+  <si>
+    <t>TC_002</t>
   </si>
   <si>
     <t>Verificar que los usuarios no puedan iniciar sesión con un correo electrónico no válido y una contraseña válida</t>
-  </si>
-  <si>
-    <t>TC_001</t>
-  </si>
-  <si>
-    <t>Pasos</t>
   </si>
   <si>
     <t>Usuario: xyz@mail.com 
@@ -61,30 +91,17 @@
 4) Haga clic en el botón de inicio de sesión</t>
   </si>
   <si>
-    <t>TC_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Navegue hasta la URL de la aplicación 
-2) Introduzca el nombre de usuario
-3) Introduzca la contraseña
-4) Haga clic en el botón de inicio de sesión </t>
-  </si>
-  <si>
-    <t>Usuario: abc@mail.com 
-Contraseña: &lt;pass&gt;</t>
-  </si>
-  <si>
-    <t>ID del caso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Debería mostrarse un mensaje de detalles de usuario no válidos. </t>
+    <t xml:space="preserve">1) Se visualiza la pantalla de Login
+2) Se visualiza el nombre de usuario
+3) Se visualiza la contraseña enmascarada
+4) Debería mostrarse un mensaje de detalles de usuario no válidos. </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -142,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -152,6 +169,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -433,66 +456,73 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:F4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="B2:F5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="18.86328125" customWidth="1"/>
-    <col min="3" max="3" width="27.796875" customWidth="1"/>
-    <col min="4" max="4" width="24.1328125" customWidth="1"/>
-    <col min="5" max="5" width="34.265625" customWidth="1"/>
-    <col min="6" max="6" width="22.1328125" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" customWidth="1"/>
+    <col min="3" max="3" width="27.85546875" customWidth="1"/>
+    <col min="4" max="4" width="24.140625" customWidth="1"/>
+    <col min="5" max="5" width="34.28515625" customWidth="1"/>
+    <col min="6" max="6" width="32.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:6">
       <c r="B2" s="3" t="s">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" ht="91.5">
+      <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>2</v>
+      <c r="E3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
-    <row r="3" spans="2:6" ht="57" x14ac:dyDescent="0.45">
-      <c r="B3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="2:6" ht="57" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:6" ht="91.5">
       <c r="B4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>14</v>
       </c>
+    </row>
+    <row r="5" spans="2:6" ht="15">
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>